<commit_message>
feat: adicionando integração com API do ClickUp
</commit_message>
<xml_diff>
--- a/demandas.xlsx
+++ b/demandas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://institutogerminare-my.sharepoint.com/personal/samuel_hironimus_institutojef_org_br/Documents/2026/Delta/Testes/sheets_automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{B383DA7F-804F-425B-BCA2-DCAA9F24DB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5CA2C36-7D19-4C2B-80A2-37B8AD64B0FC}"/>
+  <xr:revisionPtr revIDLastSave="13" documentId="8_{B383DA7F-804F-425B-BCA2-DCAA9F24DB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F484CE3-2B09-455E-AFB9-034DFFDDF0AF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2C065655-3E78-4575-8C10-12FF3694A95B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>ID</t>
   </si>
@@ -99,6 +99,21 @@
   </si>
   <si>
     <t>Descrição</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>EM PROGRESSO</t>
+  </si>
+  <si>
+    <t>Prioridade</t>
+  </si>
+  <si>
+    <t>Urgente</t>
+  </si>
+  <si>
+    <t>Baixa</t>
   </si>
 </sst>
 </file>
@@ -471,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{616A3B9B-9261-433D-833E-A1E072ED7B8A}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -482,7 +497,7 @@
     <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -504,8 +519,14 @@
       <c r="G1" t="s">
         <v>19</v>
       </c>
+      <c r="H1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" t="s">
+        <v>22</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -524,8 +545,14 @@
       <c r="F2" t="s">
         <v>18</v>
       </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -541,8 +568,14 @@
       <c r="F3">
         <v>1</v>
       </c>
+      <c r="H3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -561,8 +594,14 @@
       <c r="F4">
         <v>1</v>
       </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -580,6 +619,12 @@
       </c>
       <c r="F5">
         <v>1</v>
+      </c>
+      <c r="H5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I5" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: modularizando projeto em arquivos
</commit_message>
<xml_diff>
--- a/demandas.xlsx
+++ b/demandas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://institutogerminare-my.sharepoint.com/personal/samuel_hironimus_institutojef_org_br/Documents/2026/Delta/Testes/sheets_automation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="8_{B383DA7F-804F-425B-BCA2-DCAA9F24DB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F484CE3-2B09-455E-AFB9-034DFFDDF0AF}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{B383DA7F-804F-425B-BCA2-DCAA9F24DB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97F26FC6-1A9E-4FAB-9B98-0583C0B11592}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2C065655-3E78-4575-8C10-12FF3694A95B}"/>
   </bookViews>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
-  <si>
-    <t>ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
   <si>
     <t>Matéria</t>
   </si>
@@ -59,18 +56,6 @@
     <t>Sprint</t>
   </si>
   <si>
-    <t>BD-001</t>
-  </si>
-  <si>
-    <t>BD-002</t>
-  </si>
-  <si>
-    <t>BD-003</t>
-  </si>
-  <si>
-    <t>IA-001</t>
-  </si>
-  <si>
     <t>Bruno</t>
   </si>
   <si>
@@ -114,6 +99,18 @@
   </si>
   <si>
     <t>Baixa</t>
+  </si>
+  <si>
+    <t>Modelo conceitual</t>
+  </si>
+  <si>
+    <t>#86ahtzyhf</t>
+  </si>
+  <si>
+    <t>#86ahtzyhe</t>
+  </si>
+  <si>
+    <t>ClickUp_ID</t>
   </si>
 </sst>
 </file>
@@ -489,142 +486,142 @@
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
       <c r="G1" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1">
         <v>46171</v>
       </c>
       <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
         <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
-      </c>
-      <c r="I2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>7</v>
+      <c r="B3" t="s">
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D3" s="1">
         <v>46171</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D4" s="1">
         <v>46171</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I4" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D5" s="1">
         <v>46171</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>